<commit_message>
Regeln v1.4: Rückmeldungen der Runde, Goldenes Buch mit Archivfoto
</commit_message>
<xml_diff>
--- a/daten/saison.xlsx
+++ b/daten/saison.xlsx
@@ -1283,7 +1283,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Chaibi</t>
+          <t>Doan</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1303,10 +1303,10 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>5.5</v>
+        <v>4</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -1335,12 +1335,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Doan</t>
+          <t>E. Fernandez</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Frankfurt</t>
+          <t>Leverkusen</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1358,13 +1358,13 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>4</v>
+        <v>1.5</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -1376,7 +1376,7 @@
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -1387,12 +1387,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>E. Fernandez</t>
+          <t>Kade</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Leverkusen</t>
+          <t>Augsburg</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1407,16 +1407,16 @@
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8" t="n">
-        <v>1.5</v>
+        <v>5.5</v>
       </c>
       <c r="I8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
@@ -1428,7 +1428,7 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
Spieltag 3 ausgewertet; Webseite der Runde (docs/site) mit Wappen und Fotos
</commit_message>
<xml_diff>
--- a/daten/saison.xlsx
+++ b/daten/saison.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tabelle'!$A$1:$F$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Verlauf'!$A$1:$D$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Verlauf'!$A$1:$F$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Kategorie-Profil'!$A$1:$G$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Spieler-Beiträge'!$A$1:$N$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Spieler-Beiträge'!$A$1:$N$91</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -476,22 +476,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Sebastian</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Hallodries</t>
+          <t>Great Licors</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>23.5</v>
+        <v>39</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -509,13 +509,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>20</v>
+        <v>38.5</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -524,22 +524,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Wolfgang</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Vickings</t>
+          <t>Hallodries</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>18.5</v>
+        <v>37.5</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -548,22 +548,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Sebastian</t>
+          <t>Andreas</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Great Licors</t>
+          <t>Fischköppe</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>17.5</v>
+        <v>36</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -572,22 +572,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Andreas</t>
+          <t>Wolfgang</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Fischköppe</t>
+          <t>Vickings</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>13.5</v>
+        <v>33</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -605,13 +605,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -626,13 +626,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -648,29 +650,45 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>ST 3</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Summe</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>kum. ST 2</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>kum. ST 3</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Sebastian</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>23.5</v>
+        <v>17.5</v>
       </c>
       <c r="C2" t="n">
-        <v>23.5</v>
+        <v>21.5</v>
       </c>
       <c r="D2" t="n">
-        <v>23.5</v>
+        <v>39</v>
+      </c>
+      <c r="E2" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="F2" t="n">
+        <v>39</v>
       </c>
     </row>
     <row r="3">
@@ -683,58 +701,82 @@
         <v>20</v>
       </c>
       <c r="C3" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="D3" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="E3" t="n">
         <v>20</v>
       </c>
-      <c r="D3" t="n">
-        <v>20</v>
+      <c r="F3" t="n">
+        <v>38.5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Wolfgang</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>18.5</v>
+        <v>23.5</v>
       </c>
       <c r="C4" t="n">
-        <v>18.5</v>
+        <v>14</v>
       </c>
       <c r="D4" t="n">
-        <v>18.5</v>
+        <v>37.5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F4" t="n">
+        <v>37.5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sebastian</t>
+          <t>Andreas</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>17.5</v>
+        <v>13.5</v>
       </c>
       <c r="C5" t="n">
-        <v>17.5</v>
+        <v>22.5</v>
       </c>
       <c r="D5" t="n">
-        <v>17.5</v>
+        <v>36</v>
+      </c>
+      <c r="E5" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="F5" t="n">
+        <v>36</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Andreas</t>
+          <t>Wolfgang</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>13.5</v>
+        <v>18.5</v>
       </c>
       <c r="C6" t="n">
-        <v>13.5</v>
+        <v>14.5</v>
       </c>
       <c r="D6" t="n">
-        <v>13.5</v>
+        <v>33</v>
+      </c>
+      <c r="E6" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="F6" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="7">
@@ -747,14 +789,20 @@
         <v>12</v>
       </c>
       <c r="C7" t="n">
+        <v>14</v>
+      </c>
+      <c r="D7" t="n">
+        <v>26</v>
+      </c>
+      <c r="E7" t="n">
         <v>12</v>
       </c>
-      <c r="D7" t="n">
-        <v>12</v>
+      <c r="F7" t="n">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D7"/>
+  <autoFilter ref="A1:F7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -817,26 +865,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Sebastian</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="D2" t="n">
-        <v>5.5</v>
+        <v>7.5</v>
       </c>
       <c r="E2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G2" t="n">
-        <v>23.5</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3">
@@ -846,97 +894,97 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4.5</v>
+        <v>7.5</v>
       </c>
       <c r="C3" t="n">
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>9.5</v>
       </c>
       <c r="F3" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G3" t="n">
-        <v>20</v>
+        <v>38.5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Wolfgang</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4.5</v>
+        <v>10</v>
       </c>
       <c r="C4" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>9.5</v>
       </c>
       <c r="E4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F4" t="n">
-        <v>1.5</v>
+        <v>8</v>
       </c>
       <c r="G4" t="n">
-        <v>18.5</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sebastian</t>
+          <t>Andreas</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C5" t="n">
-        <v>4.5</v>
+        <v>10.5</v>
       </c>
       <c r="D5" t="n">
-        <v>5.5</v>
+        <v>7</v>
       </c>
       <c r="E5" t="n">
-        <v>1.5</v>
+        <v>3.5</v>
       </c>
       <c r="F5" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G5" t="n">
-        <v>17.5</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Andreas</t>
+          <t>Wolfgang</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C6" t="n">
-        <v>6</v>
+        <v>8.5</v>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E6" t="n">
-        <v>1.5</v>
+        <v>10</v>
       </c>
       <c r="F6" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="G6" t="n">
-        <v>13.5</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7">
@@ -946,22 +994,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>4.5</v>
       </c>
       <c r="C7" t="n">
-        <v>2.5</v>
+        <v>7</v>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F7" t="n">
-        <v>1.5</v>
+        <v>3.5</v>
       </c>
       <c r="G7" t="n">
-        <v>12</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -976,7 +1024,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N67"/>
+  <dimension ref="A1:N91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1089,7 +1137,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -1098,7 +1146,7 @@
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>3.5</v>
+        <v>3.25</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -1113,7 +1161,7 @@
         <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N2" t="n">
         <v>0</v>
@@ -1179,7 +1227,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Upamecano</t>
+          <t>Kim</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1202,7 +1250,7 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -1217,7 +1265,7 @@
         <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>
@@ -1231,30 +1279,30 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Bellingham</t>
+          <t>Upamecano</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Dortmund</t>
+          <t>Bayern</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -1269,7 +1317,7 @@
         <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
@@ -1283,12 +1331,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Doan</t>
+          <t>Bellingham</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Frankfurt</t>
+          <t>Dortmund</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1297,16 +1345,16 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -1335,12 +1383,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>E. Fernandez</t>
+          <t>Doan</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Leverkusen</t>
+          <t>Frankfurt</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1349,7 +1397,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -1358,13 +1406,13 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -1376,7 +1424,7 @@
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -1387,12 +1435,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Kade</t>
+          <t>E. Fernandez</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Augsburg</t>
+          <t>Leverkusen</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1401,22 +1449,22 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>5.5</v>
+        <v>2.25</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
@@ -1428,7 +1476,7 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1439,12 +1487,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Kimmich</t>
+          <t>Kade</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Augsburg</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1459,10 +1507,10 @@
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H9" t="n">
-        <v>4</v>
+        <v>5.5</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -1491,21 +1539,21 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Gregoritsch</t>
+          <t>Kimmich</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Augsburg</t>
+          <t>Bayern</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>STU</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
@@ -1514,7 +1562,7 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -1543,17 +1591,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Kane</t>
+          <t>Mohya</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Gladbach</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>STU</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -1563,10 +1611,10 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H11" t="n">
-        <v>3.5</v>
+        <v>5.5</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
@@ -1595,17 +1643,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Backhaus</t>
+          <t>Gregoritsch</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Freiburg</t>
+          <t>Augsburg</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>STU</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -1618,7 +1666,7 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
@@ -1642,26 +1690,26 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Daniel</t>
+          <t>Andreas</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Miguel</t>
+          <t>Kane</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Leverkusen</t>
+          <t>Bayern</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>STU</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
@@ -1670,46 +1718,46 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>1</v>
+        <v>3.25</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M13" t="n">
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Daniel</t>
+          <t>Andreas</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Mittelstädt</t>
+          <t>Matanovic</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Stuttgart</t>
+          <t>Freiburg</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>STU</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -1722,50 +1770,50 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Daniel</t>
+          <t>Andreas</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Vagnoman</t>
+          <t>Backhaus</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Stuttgart</t>
+          <t>Freiburg</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>
@@ -1774,22 +1822,22 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>2.5</v>
+        <v>2.75</v>
       </c>
       <c r="I15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N15" t="n">
         <v>0</v>
@@ -1803,30 +1851,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>F. Nmecha</t>
+          <t>Lukeba</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Dortmund</t>
+          <t>Leipzig</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E16" t="n">
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
@@ -1855,21 +1903,21 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Karetsas</t>
+          <t>Miguel</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Dortmund</t>
+          <t>Leverkusen</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
@@ -1878,7 +1926,7 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -1887,16 +1935,16 @@
         <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -1907,7 +1955,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Stiller</t>
+          <t>Mittelstädt</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1917,11 +1965,11 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
@@ -1930,22 +1978,22 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="I18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" t="n">
+        <v>1</v>
+      </c>
+      <c r="L18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" t="n">
         <v>3</v>
-      </c>
-      <c r="I18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M18" t="n">
-        <v>0</v>
       </c>
       <c r="N18" t="n">
         <v>0</v>
@@ -1959,17 +2007,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Tillman</t>
+          <t>Vagnoman</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Leverkusen</t>
+          <t>Stuttgart</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -1982,22 +2030,22 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N19" t="n">
         <v>0</v>
@@ -2011,12 +2059,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Wimmer</t>
+          <t>F. Nmecha</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Hoffenheim</t>
+          <t>Dortmund</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2025,22 +2073,22 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>4</v>
+        <v>3.25</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
@@ -2052,7 +2100,7 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -2063,7 +2111,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Guirassy</t>
+          <t>Karetsas</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2073,7 +2121,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>STU</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -2086,19 +2134,19 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>1.5</v>
+        <v>4</v>
       </c>
       <c r="I21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M21" t="n">
         <v>0</v>
@@ -2115,17 +2163,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Pejcinovic</t>
+          <t>S. El Mala</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Stuttgart</t>
+          <t>Köln</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>STU</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -2135,10 +2183,10 @@
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H22" t="n">
-        <v>4</v>
+        <v>5.5</v>
       </c>
       <c r="I22" t="n">
         <v>0</v>
@@ -2167,21 +2215,21 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Flekken</t>
+          <t>Stiller</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Leverkusen</t>
+          <t>Stuttgart</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
@@ -2214,35 +2262,35 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Martin</t>
+          <t>Daniel</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Diks</t>
+          <t>Tillman</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Gladbach</t>
+          <t>Leverkusen</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H24" t="n">
-        <v>4.5</v>
+        <v>4.25</v>
       </c>
       <c r="I24" t="n">
         <v>0</v>
@@ -2251,13 +2299,13 @@
         <v>0</v>
       </c>
       <c r="K24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M24" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N24" t="n">
         <v>0</v>
@@ -2266,26 +2314,26 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Martin</t>
+          <t>Daniel</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Jeltsch</t>
+          <t>Wimmer</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Stuttgart</t>
+          <t>Hoffenheim</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F25" t="n">
         <v>0</v>
@@ -2294,7 +2342,7 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>2.5</v>
+        <v>3.25</v>
       </c>
       <c r="I25" t="n">
         <v>0</v>
@@ -2303,13 +2351,13 @@
         <v>0</v>
       </c>
       <c r="K25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N25" t="n">
         <v>0</v>
@@ -2318,26 +2366,26 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Martin</t>
+          <t>Daniel</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Lienhart</t>
+          <t>Guirassy</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Freiburg</t>
+          <t>Dortmund</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>STU</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F26" t="n">
         <v>0</v>
@@ -2346,19 +2394,19 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>3.5</v>
+        <v>2</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M26" t="n">
         <v>0</v>
@@ -2370,26 +2418,26 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Martin</t>
+          <t>Daniel</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Amiri</t>
+          <t>Pejcinovic</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Mainz</t>
+          <t>Stuttgart</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>STU</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
@@ -2398,7 +2446,7 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>2</v>
+        <v>3.5</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
@@ -2422,22 +2470,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Martin</t>
+          <t>Daniel</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Burger</t>
+          <t>Flekken</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Hoffenheim</t>
+          <t>Leverkusen</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -2474,22 +2522,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Martin</t>
+          <t>Daniel</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Grönbaek</t>
+          <t>Zentner</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>HSV</t>
+          <t>Mainz</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -2502,7 +2550,7 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I29" t="n">
         <v>0</v>
@@ -2517,7 +2565,7 @@
         <v>0</v>
       </c>
       <c r="M29" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
@@ -2531,17 +2579,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Karl</t>
+          <t>Diks</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Gladbach</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -2554,22 +2602,22 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" t="n">
         <v>4</v>
-      </c>
-      <c r="I30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J30" t="n">
-        <v>0</v>
-      </c>
-      <c r="K30" t="n">
-        <v>0</v>
-      </c>
-      <c r="L30" t="n">
-        <v>0</v>
-      </c>
-      <c r="M30" t="n">
-        <v>0</v>
       </c>
       <c r="N30" t="n">
         <v>0</v>
@@ -2583,21 +2631,21 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Onyeka</t>
+          <t>Jeltsch</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Elversberg</t>
+          <t>Stuttgart</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F31" t="n">
         <v>0</v>
@@ -2606,22 +2654,22 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" t="n">
+        <v>1</v>
+      </c>
+      <c r="L31" t="n">
+        <v>1</v>
+      </c>
+      <c r="M31" t="n">
         <v>3</v>
-      </c>
-      <c r="I31" t="n">
-        <v>0</v>
-      </c>
-      <c r="J31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K31" t="n">
-        <v>0</v>
-      </c>
-      <c r="L31" t="n">
-        <v>0</v>
-      </c>
-      <c r="M31" t="n">
-        <v>0</v>
       </c>
       <c r="N31" t="n">
         <v>0</v>
@@ -2635,21 +2683,21 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Lemperle</t>
+          <t>Lienhart</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Hoffenheim</t>
+          <t>Freiburg</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>STU</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F32" t="n">
         <v>0</v>
@@ -2658,13 +2706,13 @@
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="I32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K32" t="n">
         <v>0</v>
@@ -2687,17 +2735,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Olise</t>
+          <t>Simpson-Pusey</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Köln</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>STU</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -2710,7 +2758,7 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I33" t="n">
         <v>0</v>
@@ -2725,7 +2773,7 @@
         <v>0</v>
       </c>
       <c r="M33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N33" t="n">
         <v>0</v>
@@ -2739,21 +2787,21 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Kobel</t>
+          <t>Amiri</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Dortmund</t>
+          <t>Mainz</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F34" t="n">
         <v>0</v>
@@ -2762,7 +2810,7 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="I34" t="n">
         <v>0</v>
@@ -2777,7 +2825,7 @@
         <v>0</v>
       </c>
       <c r="M34" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N34" t="n">
         <v>0</v>
@@ -2786,26 +2834,26 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Sebastian</t>
+          <t>Martin</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Laimer</t>
+          <t>Burger</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Hoffenheim</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F35" t="n">
         <v>0</v>
@@ -2814,7 +2862,7 @@
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="I35" t="n">
         <v>0</v>
@@ -2838,26 +2886,26 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Sebastian</t>
+          <t>Martin</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Ryerson</t>
+          <t>Grönbaek</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Dortmund</t>
+          <t>HSV</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F36" t="n">
         <v>0</v>
@@ -2866,7 +2914,7 @@
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
@@ -2881,7 +2929,7 @@
         <v>0</v>
       </c>
       <c r="M36" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N36" t="n">
         <v>0</v>
@@ -2890,26 +2938,26 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Sebastian</t>
+          <t>Martin</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Tapsoba</t>
+          <t>Karl</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Leverkusen</t>
+          <t>Bayern</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F37" t="n">
         <v>0</v>
@@ -2918,13 +2966,13 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="I37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K37" t="n">
         <v>0</v>
@@ -2942,17 +2990,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Sebastian</t>
+          <t>Martin</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Campbell</t>
+          <t>Leweling</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Elversberg</t>
+          <t>Stuttgart</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2967,10 +3015,10 @@
         <v>0</v>
       </c>
       <c r="G38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H38" t="n">
-        <v>3.5</v>
+        <v>5.5</v>
       </c>
       <c r="I38" t="n">
         <v>0</v>
@@ -2994,17 +3042,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Sebastian</t>
+          <t>Martin</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>El Khannouss</t>
+          <t>Onyeka</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Stuttgart</t>
+          <t>Elversberg</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -3022,13 +3070,13 @@
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K39" t="n">
         <v>0</v>
@@ -3046,22 +3094,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Sebastian</t>
+          <t>Martin</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Maza</t>
+          <t>Lemperle</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Leverkusen</t>
+          <t>Hoffenheim</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>STU</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -3074,13 +3122,13 @@
         <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="I40" t="n">
         <v>1</v>
       </c>
       <c r="J40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K40" t="n">
         <v>0</v>
@@ -3092,28 +3140,28 @@
         <v>0</v>
       </c>
       <c r="N40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Sebastian</t>
+          <t>Martin</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Pavlovic</t>
+          <t>Nkunku</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Leipzig</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>STU</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -3126,13 +3174,13 @@
         <v>0</v>
       </c>
       <c r="H41" t="n">
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="I41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J41" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K41" t="n">
         <v>0</v>
@@ -3150,26 +3198,26 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Sebastian</t>
+          <t>Martin</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Uzun</t>
+          <t>Olise</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Frankfurt</t>
+          <t>Bayern</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>STU</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F42" t="n">
         <v>0</v>
@@ -3178,7 +3226,7 @@
         <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>3.5</v>
+        <v>3.25</v>
       </c>
       <c r="I42" t="n">
         <v>0</v>
@@ -3202,26 +3250,26 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Sebastian</t>
+          <t>Martin</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Burkardt</t>
+          <t>Kobel</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Frankfurt</t>
+          <t>Dortmund</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>STU</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F43" t="n">
         <v>0</v>
@@ -3230,22 +3278,22 @@
         <v>0</v>
       </c>
       <c r="H43" t="n">
+        <v>3</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0</v>
+      </c>
+      <c r="K43" t="n">
+        <v>0</v>
+      </c>
+      <c r="L43" t="n">
+        <v>0</v>
+      </c>
+      <c r="M43" t="n">
         <v>4</v>
-      </c>
-      <c r="I43" t="n">
-        <v>1</v>
-      </c>
-      <c r="J43" t="n">
-        <v>2</v>
-      </c>
-      <c r="K43" t="n">
-        <v>0</v>
-      </c>
-      <c r="L43" t="n">
-        <v>0</v>
-      </c>
-      <c r="M43" t="n">
-        <v>0</v>
       </c>
       <c r="N43" t="n">
         <v>0</v>
@@ -3259,17 +3307,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Demirovic</t>
+          <t>Laimer</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Stuttgart</t>
+          <t>Bayern</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>STU</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -3279,16 +3327,16 @@
         <v>0</v>
       </c>
       <c r="G44" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H44" t="n">
-        <v>5.5</v>
+        <v>3.5</v>
       </c>
       <c r="I44" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K44" t="n">
         <v>0</v>
@@ -3311,17 +3359,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Neuer</t>
+          <t>Raum</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Leipzig</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -3358,12 +3406,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Sebastian</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Anton</t>
+          <t>Ryerson</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -3377,7 +3425,7 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F46" t="n">
         <v>0</v>
@@ -3386,7 +3434,7 @@
         <v>0</v>
       </c>
       <c r="H46" t="n">
-        <v>2.5</v>
+        <v>3.75</v>
       </c>
       <c r="I46" t="n">
         <v>0</v>
@@ -3395,10 +3443,10 @@
         <v>0</v>
       </c>
       <c r="K46" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L46" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M46" t="n">
         <v>2</v>
@@ -3410,12 +3458,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Sebastian</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Medina</t>
+          <t>Tapsoba</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -3429,7 +3477,7 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F47" t="n">
         <v>0</v>
@@ -3438,36 +3486,36 @@
         <v>0</v>
       </c>
       <c r="H47" t="n">
-        <v>2</v>
+        <v>2.75</v>
       </c>
       <c r="I47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M47" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Sebastian</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Quansah</t>
+          <t>Aleix Garcia</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3477,7 +3525,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E48" t="n">
@@ -3490,7 +3538,7 @@
         <v>0</v>
       </c>
       <c r="H48" t="n">
-        <v>2</v>
+        <v>3.5</v>
       </c>
       <c r="I48" t="n">
         <v>0</v>
@@ -3499,32 +3547,32 @@
         <v>0</v>
       </c>
       <c r="K48" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L48" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M48" t="n">
         <v>0</v>
       </c>
       <c r="N48" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Sebastian</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Avdullahu</t>
+          <t>Campbell</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Hoffenheim</t>
+          <t>Elversberg</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3542,13 +3590,13 @@
         <v>0</v>
       </c>
       <c r="H49" t="n">
-        <v>2</v>
+        <v>3.5</v>
       </c>
       <c r="I49" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J49" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K49" t="n">
         <v>0</v>
@@ -3566,12 +3614,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Sebastian</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Führich</t>
+          <t>El Khannouss</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -3594,13 +3642,13 @@
         <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>3.5</v>
+        <v>2</v>
       </c>
       <c r="I50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K50" t="n">
         <v>0</v>
@@ -3618,17 +3666,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Sebastian</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>M. Eggestein</t>
+          <t>Gruda</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Freiburg</t>
+          <t>Leipzig</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3646,13 +3694,13 @@
         <v>0</v>
       </c>
       <c r="H51" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="I51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K51" t="n">
         <v>0</v>
@@ -3670,17 +3718,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Sebastian</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Petkov</t>
+          <t>Maza</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Elversberg</t>
+          <t>Leverkusen</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -3689,7 +3737,7 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F52" t="n">
         <v>0</v>
@@ -3698,41 +3746,41 @@
         <v>0</v>
       </c>
       <c r="H52" t="n">
-        <v>2.5</v>
+        <v>1.75</v>
       </c>
       <c r="I52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L52" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M52" t="n">
         <v>0</v>
       </c>
       <c r="N52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Sebastian</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Prömel</t>
+          <t>Pavlovic</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Stuttgart</t>
+          <t>Bayern</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -3741,7 +3789,7 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F53" t="n">
         <v>0</v>
@@ -3750,19 +3798,19 @@
         <v>0</v>
       </c>
       <c r="H53" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="I53" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J53" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L53" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M53" t="n">
         <v>0</v>
@@ -3774,12 +3822,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Sebastian</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Ebnoutalib</t>
+          <t>Uzun</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -3789,11 +3837,11 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>STU</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F54" t="n">
         <v>0</v>
@@ -3802,41 +3850,41 @@
         <v>0</v>
       </c>
       <c r="H54" t="n">
-        <v>4.5</v>
+        <v>2.75</v>
       </c>
       <c r="I54" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J54" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M54" t="n">
         <v>0</v>
       </c>
       <c r="N54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Sebastian</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Schick</t>
+          <t>Burkardt</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Leverkusen</t>
+          <t>Frankfurt</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -3854,7 +3902,7 @@
         <v>0</v>
       </c>
       <c r="H55" t="n">
-        <v>1.5</v>
+        <v>4</v>
       </c>
       <c r="I55" t="n">
         <v>1</v>
@@ -3863,10 +3911,10 @@
         <v>2</v>
       </c>
       <c r="K55" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L55" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M55" t="n">
         <v>0</v>
@@ -3878,41 +3926,41 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Sebastian</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Atubolu</t>
+          <t>Demirovic</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Frankfurt</t>
+          <t>Stuttgart</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>STU</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F56" t="n">
         <v>0</v>
       </c>
       <c r="G56" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H56" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I56" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J56" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K56" t="n">
         <v>0</v>
@@ -3921,7 +3969,7 @@
         <v>0</v>
       </c>
       <c r="M56" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="N56" t="n">
         <v>0</v>
@@ -3930,22 +3978,22 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Wolfgang</t>
+          <t>Sebastian</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Baku</t>
+          <t>Diaby</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Leipzig</t>
+          <t>Leverkusen</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>STU</t>
         </is>
       </c>
       <c r="E57" t="n">
@@ -3958,13 +4006,13 @@
         <v>0</v>
       </c>
       <c r="H57" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="I57" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J57" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K57" t="n">
         <v>0</v>
@@ -3973,7 +4021,7 @@
         <v>0</v>
       </c>
       <c r="M57" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="N57" t="n">
         <v>0</v>
@@ -3982,12 +4030,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Wolfgang</t>
+          <t>Sebastian</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Brown</t>
+          <t>Neuer</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -3997,7 +4045,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E58" t="n">
@@ -4010,7 +4058,7 @@
         <v>0</v>
       </c>
       <c r="H58" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="I58" t="n">
         <v>0</v>
@@ -4034,12 +4082,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Wolfgang</t>
+          <t>Sebastian</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Tah</t>
+          <t>Urbig</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -4049,14 +4097,14 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E59" t="n">
         <v>1</v>
       </c>
       <c r="F59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G59" t="n">
         <v>0</v>
@@ -4077,7 +4125,7 @@
         <v>0</v>
       </c>
       <c r="M59" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N59" t="n">
         <v>0</v>
@@ -4086,26 +4134,26 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Wolfgang</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Fabio Vieira</t>
+          <t>Anton</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>HSV</t>
+          <t>Dortmund</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F60" t="n">
         <v>0</v>
@@ -4114,7 +4162,7 @@
         <v>0</v>
       </c>
       <c r="H60" t="n">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="I60" t="n">
         <v>0</v>
@@ -4123,13 +4171,13 @@
         <v>0</v>
       </c>
       <c r="K60" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L60" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M60" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N60" t="n">
         <v>0</v>
@@ -4138,26 +4186,26 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Wolfgang</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Honorat</t>
+          <t>Medina</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Gladbach</t>
+          <t>Leverkusen</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F61" t="n">
         <v>0</v>
@@ -4169,47 +4217,47 @@
         <v>2.5</v>
       </c>
       <c r="I61" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J61" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K61" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L61" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M61" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N61" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Wolfgang</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Lee</t>
+          <t>Quansah</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Mainz</t>
+          <t>Leverkusen</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F62" t="n">
         <v>0</v>
@@ -4218,7 +4266,7 @@
         <v>0</v>
       </c>
       <c r="H62" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="I62" t="n">
         <v>0</v>
@@ -4230,29 +4278,29 @@
         <v>1</v>
       </c>
       <c r="L62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M62" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Wolfgang</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Nwaneri</t>
+          <t>Avdullahu</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Dortmund</t>
+          <t>Hoffenheim</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -4270,19 +4318,19 @@
         <v>0</v>
       </c>
       <c r="H63" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L63" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M63" t="n">
         <v>0</v>
@@ -4294,17 +4342,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Wolfgang</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Suzuki</t>
+          <t>Führich</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Freiburg</t>
+          <t>Stuttgart</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -4322,7 +4370,7 @@
         <v>0</v>
       </c>
       <c r="H64" t="n">
-        <v>4.5</v>
+        <v>3.5</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -4346,22 +4394,22 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Wolfgang</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Füllkrug</t>
+          <t>Kai. Sano</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Bremen</t>
+          <t>Mainz</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>STU</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E65" t="n">
@@ -4374,13 +4422,13 @@
         <v>0</v>
       </c>
       <c r="H65" t="n">
-        <v>2</v>
+        <v>3.5</v>
       </c>
       <c r="I65" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J65" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K65" t="n">
         <v>0</v>
@@ -4398,22 +4446,22 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Wolfgang</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Mokwa</t>
+          <t>Khedira</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Elversberg</t>
+          <t>Union</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>STU</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E66" t="n">
@@ -4426,13 +4474,13 @@
         <v>0</v>
       </c>
       <c r="H66" t="n">
-        <v>2</v>
+        <v>4.5</v>
       </c>
       <c r="I66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J66" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K66" t="n">
         <v>0</v>
@@ -4450,26 +4498,26 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Wolfgang</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Vandevoordt</t>
+          <t>M. Eggestein</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Leipzig</t>
+          <t>Freiburg</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E67" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F67" t="n">
         <v>0</v>
@@ -4481,10 +4529,10 @@
         <v>2.5</v>
       </c>
       <c r="I67" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J67" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K67" t="n">
         <v>0</v>
@@ -4493,14 +4541,1262 @@
         <v>0</v>
       </c>
       <c r="M67" t="n">
+        <v>0</v>
+      </c>
+      <c r="N67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Musiala</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Bayern</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>1</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" t="n">
+        <v>4</v>
+      </c>
+      <c r="I68" t="n">
+        <v>0</v>
+      </c>
+      <c r="J68" t="n">
+        <v>0</v>
+      </c>
+      <c r="K68" t="n">
+        <v>0</v>
+      </c>
+      <c r="L68" t="n">
+        <v>0</v>
+      </c>
+      <c r="M68" t="n">
+        <v>0</v>
+      </c>
+      <c r="N68" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Petkov</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Elversberg</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>1</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I69" t="n">
+        <v>0</v>
+      </c>
+      <c r="J69" t="n">
+        <v>0</v>
+      </c>
+      <c r="K69" t="n">
+        <v>1</v>
+      </c>
+      <c r="L69" t="n">
+        <v>2</v>
+      </c>
+      <c r="M69" t="n">
+        <v>0</v>
+      </c>
+      <c r="N69" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Prömel</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>2</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" t="n">
+        <v>3</v>
+      </c>
+      <c r="I70" t="n">
+        <v>1</v>
+      </c>
+      <c r="J70" t="n">
+        <v>1</v>
+      </c>
+      <c r="K70" t="n">
+        <v>0</v>
+      </c>
+      <c r="L70" t="n">
+        <v>0</v>
+      </c>
+      <c r="M70" t="n">
+        <v>0</v>
+      </c>
+      <c r="N70" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Ebnoutalib</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Frankfurt</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>STU</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>1</v>
+      </c>
+      <c r="F71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I71" t="n">
+        <v>0</v>
+      </c>
+      <c r="J71" t="n">
+        <v>0</v>
+      </c>
+      <c r="K71" t="n">
+        <v>1</v>
+      </c>
+      <c r="L71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Schick</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Leverkusen</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>STU</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>2</v>
+      </c>
+      <c r="F72" t="n">
+        <v>0</v>
+      </c>
+      <c r="G72" t="n">
+        <v>0</v>
+      </c>
+      <c r="H72" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="I72" t="n">
+        <v>2</v>
+      </c>
+      <c r="J72" t="n">
+        <v>4</v>
+      </c>
+      <c r="K72" t="n">
+        <v>1</v>
+      </c>
+      <c r="L72" t="n">
+        <v>1</v>
+      </c>
+      <c r="M72" t="n">
+        <v>0</v>
+      </c>
+      <c r="N72" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Undav</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>STU</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>1</v>
+      </c>
+      <c r="F73" t="n">
+        <v>0</v>
+      </c>
+      <c r="G73" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" t="n">
+        <v>5</v>
+      </c>
+      <c r="I73" t="n">
+        <v>0</v>
+      </c>
+      <c r="J73" t="n">
+        <v>0</v>
+      </c>
+      <c r="K73" t="n">
+        <v>0</v>
+      </c>
+      <c r="L73" t="n">
+        <v>0</v>
+      </c>
+      <c r="M73" t="n">
+        <v>0</v>
+      </c>
+      <c r="N73" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Atubolu</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Frankfurt</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>2</v>
+      </c>
+      <c r="F74" t="n">
+        <v>0</v>
+      </c>
+      <c r="G74" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I74" t="n">
+        <v>0</v>
+      </c>
+      <c r="J74" t="n">
+        <v>0</v>
+      </c>
+      <c r="K74" t="n">
+        <v>0</v>
+      </c>
+      <c r="L74" t="n">
+        <v>0</v>
+      </c>
+      <c r="M74" t="n">
+        <v>10</v>
+      </c>
+      <c r="N74" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Wolfgang</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Baku</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>ABW</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>2</v>
+      </c>
+      <c r="F75" t="n">
+        <v>1</v>
+      </c>
+      <c r="G75" t="n">
+        <v>1</v>
+      </c>
+      <c r="H75" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I75" t="n">
+        <v>1</v>
+      </c>
+      <c r="J75" t="n">
+        <v>1</v>
+      </c>
+      <c r="K75" t="n">
+        <v>0</v>
+      </c>
+      <c r="L75" t="n">
+        <v>0</v>
+      </c>
+      <c r="M75" t="n">
+        <v>3</v>
+      </c>
+      <c r="N75" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Wolfgang</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Brown</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Bayern</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>ABW</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>1</v>
+      </c>
+      <c r="F76" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" t="n">
+        <v>0</v>
+      </c>
+      <c r="H76" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I76" t="n">
+        <v>0</v>
+      </c>
+      <c r="J76" t="n">
+        <v>0</v>
+      </c>
+      <c r="K76" t="n">
+        <v>0</v>
+      </c>
+      <c r="L76" t="n">
+        <v>0</v>
+      </c>
+      <c r="M76" t="n">
+        <v>0</v>
+      </c>
+      <c r="N76" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Wolfgang</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Schlotterbeck</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>ABW</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>1</v>
+      </c>
+      <c r="F77" t="n">
+        <v>0</v>
+      </c>
+      <c r="G77" t="n">
+        <v>0</v>
+      </c>
+      <c r="H77" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I77" t="n">
+        <v>0</v>
+      </c>
+      <c r="J77" t="n">
+        <v>0</v>
+      </c>
+      <c r="K77" t="n">
+        <v>0</v>
+      </c>
+      <c r="L77" t="n">
+        <v>0</v>
+      </c>
+      <c r="M77" t="n">
+        <v>0</v>
+      </c>
+      <c r="N77" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Wolfgang</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Svensson</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>ABW</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>1</v>
+      </c>
+      <c r="F78" t="n">
+        <v>0</v>
+      </c>
+      <c r="G78" t="n">
+        <v>0</v>
+      </c>
+      <c r="H78" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I78" t="n">
+        <v>0</v>
+      </c>
+      <c r="J78" t="n">
+        <v>0</v>
+      </c>
+      <c r="K78" t="n">
+        <v>0</v>
+      </c>
+      <c r="L78" t="n">
+        <v>0</v>
+      </c>
+      <c r="M78" t="n">
+        <v>0</v>
+      </c>
+      <c r="N78" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Wolfgang</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Tah</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Bayern</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>ABW</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>1</v>
+      </c>
+      <c r="F79" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" t="n">
+        <v>0</v>
+      </c>
+      <c r="H79" t="n">
+        <v>3</v>
+      </c>
+      <c r="I79" t="n">
+        <v>0</v>
+      </c>
+      <c r="J79" t="n">
+        <v>0</v>
+      </c>
+      <c r="K79" t="n">
+        <v>0</v>
+      </c>
+      <c r="L79" t="n">
+        <v>0</v>
+      </c>
+      <c r="M79" t="n">
+        <v>0</v>
+      </c>
+      <c r="N79" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Wolfgang</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>El Aynaoui</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>1</v>
+      </c>
+      <c r="F80" t="n">
+        <v>0</v>
+      </c>
+      <c r="G80" t="n">
+        <v>0</v>
+      </c>
+      <c r="H80" t="n">
+        <v>3</v>
+      </c>
+      <c r="I80" t="n">
+        <v>0</v>
+      </c>
+      <c r="J80" t="n">
+        <v>0</v>
+      </c>
+      <c r="K80" t="n">
+        <v>0</v>
+      </c>
+      <c r="L80" t="n">
+        <v>0</v>
+      </c>
+      <c r="M80" t="n">
+        <v>0</v>
+      </c>
+      <c r="N80" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Wolfgang</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Fabio Vieira</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>HSV</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>1</v>
+      </c>
+      <c r="F81" t="n">
+        <v>0</v>
+      </c>
+      <c r="G81" t="n">
+        <v>0</v>
+      </c>
+      <c r="H81" t="n">
+        <v>5</v>
+      </c>
+      <c r="I81" t="n">
+        <v>0</v>
+      </c>
+      <c r="J81" t="n">
+        <v>0</v>
+      </c>
+      <c r="K81" t="n">
+        <v>0</v>
+      </c>
+      <c r="L81" t="n">
+        <v>0</v>
+      </c>
+      <c r="M81" t="n">
+        <v>0</v>
+      </c>
+      <c r="N81" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Wolfgang</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Honorat</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Gladbach</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>1</v>
+      </c>
+      <c r="F82" t="n">
+        <v>0</v>
+      </c>
+      <c r="G82" t="n">
+        <v>0</v>
+      </c>
+      <c r="H82" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I82" t="n">
+        <v>0</v>
+      </c>
+      <c r="J82" t="n">
+        <v>0</v>
+      </c>
+      <c r="K82" t="n">
+        <v>2</v>
+      </c>
+      <c r="L82" t="n">
+        <v>4</v>
+      </c>
+      <c r="M82" t="n">
+        <v>0</v>
+      </c>
+      <c r="N82" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Wolfgang</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Lee</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Mainz</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>2</v>
+      </c>
+      <c r="F83" t="n">
+        <v>0</v>
+      </c>
+      <c r="G83" t="n">
+        <v>0</v>
+      </c>
+      <c r="H83" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I83" t="n">
+        <v>0</v>
+      </c>
+      <c r="J83" t="n">
+        <v>0</v>
+      </c>
+      <c r="K83" t="n">
+        <v>1</v>
+      </c>
+      <c r="L83" t="n">
+        <v>2</v>
+      </c>
+      <c r="M83" t="n">
+        <v>0</v>
+      </c>
+      <c r="N83" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Wolfgang</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Nwaneri</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>2</v>
+      </c>
+      <c r="F84" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="I84" t="n">
+        <v>0</v>
+      </c>
+      <c r="J84" t="n">
+        <v>0</v>
+      </c>
+      <c r="K84" t="n">
+        <v>1</v>
+      </c>
+      <c r="L84" t="n">
+        <v>2</v>
+      </c>
+      <c r="M84" t="n">
+        <v>0</v>
+      </c>
+      <c r="N84" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Wolfgang</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Suzuki</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Freiburg</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>2</v>
+      </c>
+      <c r="F85" t="n">
+        <v>0</v>
+      </c>
+      <c r="G85" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="I85" t="n">
+        <v>0</v>
+      </c>
+      <c r="J85" t="n">
+        <v>0</v>
+      </c>
+      <c r="K85" t="n">
+        <v>0</v>
+      </c>
+      <c r="L85" t="n">
+        <v>0</v>
+      </c>
+      <c r="M85" t="n">
+        <v>0</v>
+      </c>
+      <c r="N85" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Wolfgang</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Veerman</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>1</v>
+      </c>
+      <c r="F86" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" t="n">
+        <v>3</v>
+      </c>
+      <c r="I86" t="n">
+        <v>0</v>
+      </c>
+      <c r="J86" t="n">
+        <v>0</v>
+      </c>
+      <c r="K86" t="n">
+        <v>0</v>
+      </c>
+      <c r="L86" t="n">
+        <v>0</v>
+      </c>
+      <c r="M86" t="n">
+        <v>0</v>
+      </c>
+      <c r="N86" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Wolfgang</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Füllkrug</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Bremen</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>STU</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>1</v>
+      </c>
+      <c r="F87" t="n">
+        <v>0</v>
+      </c>
+      <c r="G87" t="n">
+        <v>0</v>
+      </c>
+      <c r="H87" t="n">
+        <v>2</v>
+      </c>
+      <c r="I87" t="n">
+        <v>1</v>
+      </c>
+      <c r="J87" t="n">
+        <v>2</v>
+      </c>
+      <c r="K87" t="n">
+        <v>0</v>
+      </c>
+      <c r="L87" t="n">
+        <v>0</v>
+      </c>
+      <c r="M87" t="n">
+        <v>0</v>
+      </c>
+      <c r="N87" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Wolfgang</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Luis Diaz</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Bayern</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>STU</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>1</v>
+      </c>
+      <c r="F88" t="n">
+        <v>0</v>
+      </c>
+      <c r="G88" t="n">
+        <v>0</v>
+      </c>
+      <c r="H88" t="n">
+        <v>4</v>
+      </c>
+      <c r="I88" t="n">
+        <v>0</v>
+      </c>
+      <c r="J88" t="n">
+        <v>0</v>
+      </c>
+      <c r="K88" t="n">
+        <v>0</v>
+      </c>
+      <c r="L88" t="n">
+        <v>0</v>
+      </c>
+      <c r="M88" t="n">
+        <v>0</v>
+      </c>
+      <c r="N88" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Wolfgang</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Mokwa</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Elversberg</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>STU</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>1</v>
+      </c>
+      <c r="F89" t="n">
+        <v>0</v>
+      </c>
+      <c r="G89" t="n">
+        <v>0</v>
+      </c>
+      <c r="H89" t="n">
+        <v>2</v>
+      </c>
+      <c r="I89" t="n">
+        <v>1</v>
+      </c>
+      <c r="J89" t="n">
+        <v>2</v>
+      </c>
+      <c r="K89" t="n">
+        <v>0</v>
+      </c>
+      <c r="L89" t="n">
+        <v>0</v>
+      </c>
+      <c r="M89" t="n">
+        <v>0</v>
+      </c>
+      <c r="N89" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Wolfgang</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Saibari</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Bayern</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>STU</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>1</v>
+      </c>
+      <c r="F90" t="n">
+        <v>0</v>
+      </c>
+      <c r="G90" t="n">
+        <v>0</v>
+      </c>
+      <c r="H90" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I90" t="n">
+        <v>0</v>
+      </c>
+      <c r="J90" t="n">
+        <v>0</v>
+      </c>
+      <c r="K90" t="n">
+        <v>1</v>
+      </c>
+      <c r="L90" t="n">
+        <v>1</v>
+      </c>
+      <c r="M90" t="n">
+        <v>0</v>
+      </c>
+      <c r="N90" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Wolfgang</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Vandevoordt</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>2</v>
+      </c>
+      <c r="F91" t="n">
+        <v>0</v>
+      </c>
+      <c r="G91" t="n">
+        <v>0</v>
+      </c>
+      <c r="H91" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I91" t="n">
+        <v>0</v>
+      </c>
+      <c r="J91" t="n">
+        <v>0</v>
+      </c>
+      <c r="K91" t="n">
+        <v>0</v>
+      </c>
+      <c r="L91" t="n">
+        <v>0</v>
+      </c>
+      <c r="M91" t="n">
         <v>6</v>
       </c>
-      <c r="N67" t="n">
+      <c r="N91" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N67"/>
+  <autoFilter ref="A1:N91"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Spieltag 4 ausgewertet; Regeln v1.5 (Jugendspieler, Einsatz und Auszahlung); Kasse auf der Seite
</commit_message>
<xml_diff>
--- a/daten/saison.xlsx
+++ b/daten/saison.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tabelle'!$A$1:$F$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Verlauf'!$A$1:$F$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Verlauf'!$A$1:$H$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Kategorie-Profil'!$A$1:$G$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Spieler-Beiträge'!$A$1:$N$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Spieler-Beiträge'!$A$1:$N$99</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -476,22 +476,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Sebastian</t>
+          <t>Andreas</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Great Licors</t>
+          <t>Fischköppe</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>39</v>
+        <v>62.5</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -509,13 +509,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>38.5</v>
+        <v>56</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -524,22 +524,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Sebastian</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Hallodries</t>
+          <t>Great Licors</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>37.5</v>
+        <v>55.5</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -548,22 +548,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Andreas</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Fischköppe</t>
+          <t>Hallodries</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -581,13 +581,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -605,13 +605,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -635,6 +635,8 @@
     <col width="7" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
     <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -655,40 +657,56 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>ST 4</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Summe</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>kum. ST 2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>kum. ST 3</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>kum. ST 4</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sebastian</t>
+          <t>Andreas</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>17.5</v>
+        <v>13.5</v>
       </c>
       <c r="C2" t="n">
-        <v>21.5</v>
+        <v>22.5</v>
       </c>
       <c r="D2" t="n">
-        <v>39</v>
+        <v>26.5</v>
       </c>
       <c r="E2" t="n">
-        <v>17.5</v>
+        <v>62.5</v>
       </c>
       <c r="F2" t="n">
-        <v>39</v>
+        <v>13.5</v>
+      </c>
+      <c r="G2" t="n">
+        <v>36</v>
+      </c>
+      <c r="H2" t="n">
+        <v>62.5</v>
       </c>
     </row>
     <row r="3">
@@ -704,57 +722,75 @@
         <v>18.5</v>
       </c>
       <c r="D3" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>56</v>
+      </c>
+      <c r="F3" t="n">
+        <v>20</v>
+      </c>
+      <c r="G3" t="n">
         <v>38.5</v>
       </c>
-      <c r="E3" t="n">
-        <v>20</v>
-      </c>
-      <c r="F3" t="n">
-        <v>38.5</v>
+      <c r="H3" t="n">
+        <v>56</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Sebastian</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>23.5</v>
+        <v>17.5</v>
       </c>
       <c r="C4" t="n">
-        <v>14</v>
+        <v>21.5</v>
       </c>
       <c r="D4" t="n">
-        <v>37.5</v>
+        <v>16.5</v>
       </c>
       <c r="E4" t="n">
-        <v>23.5</v>
+        <v>55.5</v>
       </c>
       <c r="F4" t="n">
-        <v>37.5</v>
+        <v>17.5</v>
+      </c>
+      <c r="G4" t="n">
+        <v>39</v>
+      </c>
+      <c r="H4" t="n">
+        <v>55.5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Andreas</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>13.5</v>
+        <v>23.5</v>
       </c>
       <c r="C5" t="n">
-        <v>22.5</v>
+        <v>14</v>
       </c>
       <c r="D5" t="n">
-        <v>36</v>
+        <v>14.5</v>
       </c>
       <c r="E5" t="n">
-        <v>13.5</v>
+        <v>52</v>
       </c>
       <c r="F5" t="n">
-        <v>36</v>
+        <v>23.5</v>
+      </c>
+      <c r="G5" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="H5" t="n">
+        <v>52</v>
       </c>
     </row>
     <row r="6">
@@ -770,13 +806,19 @@
         <v>14.5</v>
       </c>
       <c r="D6" t="n">
+        <v>12</v>
+      </c>
+      <c r="E6" t="n">
+        <v>45</v>
+      </c>
+      <c r="F6" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="G6" t="n">
         <v>33</v>
       </c>
-      <c r="E6" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="F6" t="n">
-        <v>33</v>
+      <c r="H6" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="7">
@@ -792,17 +834,23 @@
         <v>14</v>
       </c>
       <c r="D7" t="n">
+        <v>18</v>
+      </c>
+      <c r="E7" t="n">
+        <v>44</v>
+      </c>
+      <c r="F7" t="n">
+        <v>12</v>
+      </c>
+      <c r="G7" t="n">
         <v>26</v>
       </c>
-      <c r="E7" t="n">
-        <v>12</v>
-      </c>
-      <c r="F7" t="n">
-        <v>26</v>
+      <c r="H7" t="n">
+        <v>44</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F7"/>
+  <autoFilter ref="A1:H7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -865,26 +913,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sebastian</t>
+          <t>Andreas</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C2" t="n">
-        <v>7.5</v>
+        <v>14.5</v>
       </c>
       <c r="D2" t="n">
-        <v>7.5</v>
+        <v>12</v>
       </c>
       <c r="E2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F2" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="G2" t="n">
-        <v>39</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="3">
@@ -894,72 +942,72 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7.5</v>
+        <v>11.5</v>
       </c>
       <c r="C3" t="n">
-        <v>5.5</v>
+        <v>10.5</v>
       </c>
       <c r="D3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E3" t="n">
-        <v>9.5</v>
+        <v>12.5</v>
       </c>
       <c r="F3" t="n">
-        <v>9</v>
+        <v>13.5</v>
       </c>
       <c r="G3" t="n">
-        <v>38.5</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Sebastian</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C4" t="n">
-        <v>3</v>
+        <v>13.5</v>
       </c>
       <c r="D4" t="n">
         <v>9.5</v>
       </c>
       <c r="E4" t="n">
-        <v>7</v>
+        <v>8.5</v>
       </c>
       <c r="F4" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G4" t="n">
-        <v>37.5</v>
+        <v>55.5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Andreas</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="B5" t="n">
+        <v>12</v>
+      </c>
+      <c r="C5" t="n">
         <v>6</v>
       </c>
-      <c r="C5" t="n">
-        <v>10.5</v>
-      </c>
       <c r="D5" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E5" t="n">
-        <v>3.5</v>
+        <v>11</v>
       </c>
       <c r="F5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G5" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6">
@@ -969,22 +1017,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C6" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="D6" t="n">
         <v>8.5</v>
       </c>
-      <c r="D6" t="n">
-        <v>5</v>
-      </c>
       <c r="E6" t="n">
-        <v>10</v>
+        <v>11.5</v>
       </c>
       <c r="F6" t="n">
-        <v>3.5</v>
+        <v>5.5</v>
       </c>
       <c r="G6" t="n">
-        <v>33</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7">
@@ -994,22 +1042,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
       <c r="C7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D7" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E7" t="n">
-        <v>5</v>
+        <v>10.5</v>
       </c>
       <c r="F7" t="n">
-        <v>3.5</v>
+        <v>8</v>
       </c>
       <c r="G7" t="n">
-        <v>26</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -1024,7 +1072,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N91"/>
+  <dimension ref="A1:N99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1137,7 +1185,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -1146,7 +1194,7 @@
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>3.25</v>
+        <v>2.83</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -1155,10 +1203,10 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M2" t="n">
         <v>1</v>
@@ -1279,7 +1327,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Upamecano</t>
+          <t>Stanisic</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1293,7 +1341,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -1302,7 +1350,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -1317,10 +1365,10 @@
         <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -1331,30 +1379,30 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Bellingham</t>
+          <t>Upamecano</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Dortmund</t>
+          <t>Bayern</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>3.5</v>
+        <v>3.17</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -1369,7 +1417,7 @@
         <v>0</v>
       </c>
       <c r="M6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N6" t="n">
         <v>0</v>
@@ -1383,12 +1431,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Doan</t>
+          <t>Bellingham</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Frankfurt</t>
+          <t>Dortmund</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1397,16 +1445,16 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>3</v>
+        <v>3.17</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -1415,10 +1463,10 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M7" t="n">
         <v>0</v>
@@ -1435,12 +1483,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>E. Fernandez</t>
+          <t>Doan</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Leverkusen</t>
+          <t>Frankfurt</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1449,7 +1497,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -1458,25 +1506,25 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>2.25</v>
+        <v>3</v>
       </c>
       <c r="I8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M8" t="n">
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1487,12 +1535,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Kade</t>
+          <t>E. Fernandez</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Augsburg</t>
+          <t>Leverkusen</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1501,22 +1549,22 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>5.5</v>
+        <v>2.5</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -1528,7 +1576,7 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1539,12 +1587,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Kimmich</t>
+          <t>Kade</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Augsburg</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1553,16 +1601,16 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H10" t="n">
-        <v>3.5</v>
+        <v>5.5</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -1591,12 +1639,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Mohya</t>
+          <t>Kimmich</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Gladbach</t>
+          <t>Bayern</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1605,16 +1653,16 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>5.5</v>
+        <v>3</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
@@ -1643,30 +1691,30 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Gregoritsch</t>
+          <t>Mohya</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Augsburg</t>
+          <t>Gladbach</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>STU</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H12" t="n">
-        <v>4</v>
+        <v>4.75</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
@@ -1695,12 +1743,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Kane</t>
+          <t>Gregoritsch</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Augsburg</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1709,7 +1757,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
@@ -1718,13 +1766,13 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>3.25</v>
+        <v>4</v>
       </c>
       <c r="I13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
@@ -1747,12 +1795,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Matanovic</t>
+          <t>Kane</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Freiburg</t>
+          <t>Bayern</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1761,7 +1809,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
@@ -1770,13 +1818,13 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>1</v>
+        <v>2.83</v>
       </c>
       <c r="I14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J14" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
@@ -1799,7 +1847,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Backhaus</t>
+          <t>Matanovic</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1809,7 +1857,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>STU</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -1822,13 +1870,13 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>2.75</v>
+        <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -1840,32 +1888,32 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Daniel</t>
+          <t>Andreas</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Lukeba</t>
+          <t>Backhaus</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Leipzig</t>
+          <t>Freiburg</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
@@ -1874,22 +1922,22 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="n">
         <v>4</v>
-      </c>
-      <c r="I16" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" t="n">
-        <v>0</v>
       </c>
       <c r="N16" t="n">
         <v>0</v>
@@ -1903,12 +1951,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Miguel</t>
+          <t>Lukeba</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Leverkusen</t>
+          <t>Leipzig</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1917,7 +1965,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
@@ -1926,7 +1974,7 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -1935,16 +1983,16 @@
         <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -1955,12 +2003,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Mittelstädt</t>
+          <t>Miguel</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Stuttgart</t>
+          <t>Leverkusen</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1969,7 +2017,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
@@ -1978,7 +2026,7 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>2.75</v>
+        <v>1.83</v>
       </c>
       <c r="I18" t="n">
         <v>1</v>
@@ -1987,16 +2035,16 @@
         <v>1</v>
       </c>
       <c r="K18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
@@ -2007,7 +2055,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Vagnoman</t>
+          <t>Mittelstädt</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2021,7 +2069,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
@@ -2030,7 +2078,7 @@
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>2.5</v>
+        <v>3.17</v>
       </c>
       <c r="I19" t="n">
         <v>1</v>
@@ -2045,7 +2093,7 @@
         <v>1</v>
       </c>
       <c r="M19" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N19" t="n">
         <v>0</v>
@@ -2059,17 +2107,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>F. Nmecha</t>
+          <t>Vagnoman</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Dortmund</t>
+          <t>Stuttgart</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -2082,25 +2130,25 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>3.25</v>
+        <v>3</v>
       </c>
       <c r="I20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -2111,7 +2159,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Karetsas</t>
+          <t>F. Nmecha</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2125,22 +2173,22 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>4</v>
+        <v>2.83</v>
       </c>
       <c r="I21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
@@ -2152,7 +2200,7 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -2163,12 +2211,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>S. El Mala</t>
+          <t>Karaman</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Köln</t>
+          <t>Schalke</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2183,10 +2231,10 @@
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>5.5</v>
+        <v>3.5</v>
       </c>
       <c r="I22" t="n">
         <v>0</v>
@@ -2215,12 +2263,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Stiller</t>
+          <t>Karetsas</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Stuttgart</t>
+          <t>Dortmund</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2238,7 +2286,7 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="I23" t="n">
         <v>0</v>
@@ -2267,12 +2315,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Tillman</t>
+          <t>S. El Mala</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Leverkusen</t>
+          <t>Köln</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2290,7 +2338,7 @@
         <v>1</v>
       </c>
       <c r="H24" t="n">
-        <v>4.25</v>
+        <v>4.5</v>
       </c>
       <c r="I24" t="n">
         <v>0</v>
@@ -2299,10 +2347,10 @@
         <v>0</v>
       </c>
       <c r="K24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M24" t="n">
         <v>0</v>
@@ -2319,12 +2367,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Wimmer</t>
+          <t>Stiller</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Hoffenheim</t>
+          <t>Stuttgart</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2342,7 +2390,7 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>3.25</v>
+        <v>3</v>
       </c>
       <c r="I25" t="n">
         <v>0</v>
@@ -2371,17 +2419,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Guirassy</t>
+          <t>Tillman</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Dortmund</t>
+          <t>Leverkusen</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>STU</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -2391,19 +2439,19 @@
         <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H26" t="n">
-        <v>2</v>
+        <v>4.25</v>
       </c>
       <c r="I26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L26" t="n">
         <v>2</v>
@@ -2423,21 +2471,21 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Pejcinovic</t>
+          <t>Wimmer</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Stuttgart</t>
+          <t>Hoffenheim</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>STU</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
@@ -2446,7 +2494,7 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>3.5</v>
+        <v>3.33</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
@@ -2475,21 +2523,21 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Flekken</t>
+          <t>Guirassy</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Leverkusen</t>
+          <t>Dortmund</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>STU</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F28" t="n">
         <v>0</v>
@@ -2498,19 +2546,19 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>3</v>
+        <v>2.67</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J28" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K28" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L28" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M28" t="n">
         <v>0</v>
@@ -2527,21 +2575,21 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Zentner</t>
+          <t>Pejcinovic</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Mainz</t>
+          <t>Stuttgart</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>STU</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F29" t="n">
         <v>0</v>
@@ -2550,7 +2598,7 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="I29" t="n">
         <v>0</v>
@@ -2565,7 +2613,7 @@
         <v>0</v>
       </c>
       <c r="M29" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
@@ -2574,22 +2622,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Martin</t>
+          <t>Daniel</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Diks</t>
+          <t>Romulo</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Gladbach</t>
+          <t>Leipzig</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>STU</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -2602,7 +2650,7 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="I30" t="n">
         <v>0</v>
@@ -2617,7 +2665,7 @@
         <v>0</v>
       </c>
       <c r="M30" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N30" t="n">
         <v>0</v>
@@ -2626,22 +2674,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Martin</t>
+          <t>Daniel</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Jeltsch</t>
+          <t>Flekken</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Stuttgart</t>
+          <t>Leverkusen</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -2654,7 +2702,7 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="I31" t="n">
         <v>0</v>
@@ -2663,13 +2711,13 @@
         <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M31" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="N31" t="n">
         <v>0</v>
@@ -2678,26 +2726,26 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Martin</t>
+          <t>Daniel</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Lienhart</t>
+          <t>Zentner</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Freiburg</t>
+          <t>Mainz</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F32" t="n">
         <v>0</v>
@@ -2721,7 +2769,7 @@
         <v>0</v>
       </c>
       <c r="M32" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N32" t="n">
         <v>0</v>
@@ -2735,12 +2783,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Simpson-Pusey</t>
+          <t>Diks</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Köln</t>
+          <t>Gladbach</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2749,7 +2797,7 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F33" t="n">
         <v>0</v>
@@ -2758,7 +2806,7 @@
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>4</v>
+        <v>4.75</v>
       </c>
       <c r="I33" t="n">
         <v>0</v>
@@ -2773,7 +2821,7 @@
         <v>0</v>
       </c>
       <c r="M33" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="N33" t="n">
         <v>0</v>
@@ -2787,17 +2835,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Amiri</t>
+          <t>Jeltsch</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Mainz</t>
+          <t>Stuttgart</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -2810,7 +2858,7 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>3.5</v>
+        <v>2.75</v>
       </c>
       <c r="I34" t="n">
         <v>0</v>
@@ -2819,13 +2867,13 @@
         <v>0</v>
       </c>
       <c r="K34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N34" t="n">
         <v>0</v>
@@ -2839,21 +2887,21 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Burger</t>
+          <t>Lienhart</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Hoffenheim</t>
+          <t>Freiburg</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F35" t="n">
         <v>0</v>
@@ -2862,7 +2910,7 @@
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="I35" t="n">
         <v>0</v>
@@ -2877,7 +2925,7 @@
         <v>0</v>
       </c>
       <c r="M35" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N35" t="n">
         <v>0</v>
@@ -2891,17 +2939,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Grönbaek</t>
+          <t>Simpson-Pusey</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>HSV</t>
+          <t>Köln</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -2914,7 +2962,7 @@
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>4.5</v>
+        <v>4.25</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
@@ -2929,7 +2977,7 @@
         <v>0</v>
       </c>
       <c r="M36" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N36" t="n">
         <v>0</v>
@@ -2943,12 +2991,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Karl</t>
+          <t>Amiri</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Mainz</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2957,7 +3005,7 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F37" t="n">
         <v>0</v>
@@ -2969,10 +3017,10 @@
         <v>3.5</v>
       </c>
       <c r="I37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K37" t="n">
         <v>0</v>
@@ -2995,12 +3043,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Leweling</t>
+          <t>Burger</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Stuttgart</t>
+          <t>Hoffenheim</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -3009,16 +3057,16 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F38" t="n">
         <v>0</v>
       </c>
       <c r="G38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>5.5</v>
+        <v>3</v>
       </c>
       <c r="I38" t="n">
         <v>0</v>
@@ -3047,12 +3095,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Onyeka</t>
+          <t>Grönbaek</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Elversberg</t>
+          <t>HSV</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -3061,7 +3109,7 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F39" t="n">
         <v>0</v>
@@ -3070,7 +3118,7 @@
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>3</v>
+        <v>3.83</v>
       </c>
       <c r="I39" t="n">
         <v>0</v>
@@ -3079,10 +3127,10 @@
         <v>0</v>
       </c>
       <c r="K39" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L39" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M39" t="n">
         <v>0</v>
@@ -3099,21 +3147,21 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Lemperle</t>
+          <t>Karl</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Hoffenheim</t>
+          <t>Bayern</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>STU</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F40" t="n">
         <v>0</v>
@@ -3122,13 +3170,13 @@
         <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>1.5</v>
+        <v>3.5</v>
       </c>
       <c r="I40" t="n">
         <v>1</v>
       </c>
       <c r="J40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K40" t="n">
         <v>0</v>
@@ -3151,36 +3199,36 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Nkunku</t>
+          <t>Leweling</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Leipzig</t>
+          <t>Stuttgart</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>STU</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F41" t="n">
         <v>0</v>
       </c>
       <c r="G41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H41" t="n">
-        <v>2.5</v>
+        <v>4.5</v>
       </c>
       <c r="I41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K41" t="n">
         <v>0</v>
@@ -3203,30 +3251,30 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Olise</t>
+          <t>Onyeka</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Elversberg</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>STU</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E42" t="n">
         <v>2</v>
       </c>
       <c r="F42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H42" t="n">
-        <v>3.25</v>
+        <v>4.25</v>
       </c>
       <c r="I42" t="n">
         <v>0</v>
@@ -3255,17 +3303,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Kobel</t>
+          <t>Lemperle</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Dortmund</t>
+          <t>Hoffenheim</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>STU</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -3281,10 +3329,10 @@
         <v>3</v>
       </c>
       <c r="I43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J43" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K43" t="n">
         <v>0</v>
@@ -3293,7 +3341,7 @@
         <v>0</v>
       </c>
       <c r="M43" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N43" t="n">
         <v>0</v>
@@ -3302,22 +3350,22 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Sebastian</t>
+          <t>Martin</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Laimer</t>
+          <t>Nkunku</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Leipzig</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>STU</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -3330,13 +3378,13 @@
         <v>0</v>
       </c>
       <c r="H44" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="I44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J44" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K44" t="n">
         <v>0</v>
@@ -3354,26 +3402,26 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Sebastian</t>
+          <t>Martin</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Raum</t>
+          <t>Olise</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Leipzig</t>
+          <t>Bayern</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>STU</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F45" t="n">
         <v>0</v>
@@ -3382,36 +3430,36 @@
         <v>0</v>
       </c>
       <c r="H45" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="I45" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J45" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="K45" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L45" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M45" t="n">
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Sebastian</t>
+          <t>Martin</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Ryerson</t>
+          <t>Kobel</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -3421,11 +3469,11 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F46" t="n">
         <v>0</v>
@@ -3434,7 +3482,7 @@
         <v>0</v>
       </c>
       <c r="H46" t="n">
-        <v>3.75</v>
+        <v>2.83</v>
       </c>
       <c r="I46" t="n">
         <v>0</v>
@@ -3449,7 +3497,7 @@
         <v>0</v>
       </c>
       <c r="M46" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N46" t="n">
         <v>0</v>
@@ -3463,12 +3511,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Tapsoba</t>
+          <t>Gadou</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Leverkusen</t>
+          <t>Dortmund</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -3477,16 +3525,16 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G47" t="n">
         <v>0</v>
       </c>
       <c r="H47" t="n">
-        <v>2.75</v>
+        <v>4</v>
       </c>
       <c r="I47" t="n">
         <v>0</v>
@@ -3495,13 +3543,13 @@
         <v>0</v>
       </c>
       <c r="K47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M47" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N47" t="n">
         <v>0</v>
@@ -3515,17 +3563,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Aleix Garcia</t>
+          <t>Laimer</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Leverkusen</t>
+          <t>Bayern</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E48" t="n">
@@ -3567,17 +3615,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Campbell</t>
+          <t>Raum</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Elversberg</t>
+          <t>Leipzig</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E49" t="n">
@@ -3590,7 +3638,7 @@
         <v>0</v>
       </c>
       <c r="H49" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="I49" t="n">
         <v>0</v>
@@ -3619,21 +3667,21 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>El Khannouss</t>
+          <t>Ryerson</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Stuttgart</t>
+          <t>Dortmund</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F50" t="n">
         <v>0</v>
@@ -3642,13 +3690,13 @@
         <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>2</v>
+        <v>3.5</v>
       </c>
       <c r="I50" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J50" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K50" t="n">
         <v>0</v>
@@ -3657,7 +3705,7 @@
         <v>0</v>
       </c>
       <c r="M50" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N50" t="n">
         <v>0</v>
@@ -3671,21 +3719,21 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Gruda</t>
+          <t>Tapsoba</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Leipzig</t>
+          <t>Leverkusen</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F51" t="n">
         <v>0</v>
@@ -3694,7 +3742,7 @@
         <v>0</v>
       </c>
       <c r="H51" t="n">
-        <v>2</v>
+        <v>2.67</v>
       </c>
       <c r="I51" t="n">
         <v>0</v>
@@ -3703,13 +3751,13 @@
         <v>0</v>
       </c>
       <c r="K51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M51" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N51" t="n">
         <v>0</v>
@@ -3723,7 +3771,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Maza</t>
+          <t>Aleix Garcia</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -3746,13 +3794,13 @@
         <v>0</v>
       </c>
       <c r="H52" t="n">
-        <v>1.75</v>
+        <v>3</v>
       </c>
       <c r="I52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K52" t="n">
         <v>0</v>
@@ -3764,7 +3812,7 @@
         <v>0</v>
       </c>
       <c r="N52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -3775,12 +3823,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Pavlovic</t>
+          <t>Campbell</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Elversberg</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -3789,7 +3837,7 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F53" t="n">
         <v>0</v>
@@ -3807,10 +3855,10 @@
         <v>0</v>
       </c>
       <c r="K53" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L53" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M53" t="n">
         <v>0</v>
@@ -3827,12 +3875,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Uzun</t>
+          <t>El Khannouss</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Frankfurt</t>
+          <t>Stuttgart</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -3841,7 +3889,7 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F54" t="n">
         <v>0</v>
@@ -3850,13 +3898,13 @@
         <v>0</v>
       </c>
       <c r="H54" t="n">
-        <v>2.75</v>
+        <v>2</v>
       </c>
       <c r="I54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K54" t="n">
         <v>0</v>
@@ -3868,7 +3916,7 @@
         <v>0</v>
       </c>
       <c r="N54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
@@ -3879,21 +3927,21 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Burkardt</t>
+          <t>Gruda</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Frankfurt</t>
+          <t>Leipzig</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>STU</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F55" t="n">
         <v>0</v>
@@ -3902,13 +3950,13 @@
         <v>0</v>
       </c>
       <c r="H55" t="n">
-        <v>4</v>
+        <v>2.75</v>
       </c>
       <c r="I55" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J55" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K55" t="n">
         <v>0</v>
@@ -3931,36 +3979,36 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Demirovic</t>
+          <t>Maza</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Stuttgart</t>
+          <t>Leverkusen</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>STU</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F56" t="n">
         <v>0</v>
       </c>
       <c r="G56" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H56" t="n">
-        <v>4</v>
+        <v>2.17</v>
       </c>
       <c r="I56" t="n">
         <v>1</v>
       </c>
       <c r="J56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K56" t="n">
         <v>0</v>
@@ -3972,7 +4020,7 @@
         <v>0</v>
       </c>
       <c r="N56" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57">
@@ -3983,21 +4031,21 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Diaby</t>
+          <t>Pavlovic</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Leverkusen</t>
+          <t>Bayern</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>STU</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F57" t="n">
         <v>0</v>
@@ -4006,7 +4054,7 @@
         <v>0</v>
       </c>
       <c r="H57" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I57" t="n">
         <v>0</v>
@@ -4015,10 +4063,10 @@
         <v>0</v>
       </c>
       <c r="K57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L57" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M57" t="n">
         <v>0</v>
@@ -4035,21 +4083,21 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Neuer</t>
+          <t>Uzun</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Frankfurt</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F58" t="n">
         <v>0</v>
@@ -4061,10 +4109,10 @@
         <v>3</v>
       </c>
       <c r="I58" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J58" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K58" t="n">
         <v>0</v>
@@ -4076,7 +4124,7 @@
         <v>0</v>
       </c>
       <c r="N58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59">
@@ -4087,24 +4135,24 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Urbig</t>
+          <t>Burkardt</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Frankfurt</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>STU</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F59" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G59" t="n">
         <v>0</v>
@@ -4113,10 +4161,10 @@
         <v>3</v>
       </c>
       <c r="I59" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J59" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K59" t="n">
         <v>0</v>
@@ -4125,7 +4173,7 @@
         <v>0</v>
       </c>
       <c r="M59" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N59" t="n">
         <v>0</v>
@@ -4134,22 +4182,22 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Sebastian</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Anton</t>
+          <t>Demirovic</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Dortmund</t>
+          <t>Stuttgart</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>STU</t>
         </is>
       </c>
       <c r="E60" t="n">
@@ -4159,25 +4207,25 @@
         <v>0</v>
       </c>
       <c r="G60" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H60" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="I60" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J60" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K60" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L60" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M60" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N60" t="n">
         <v>0</v>
@@ -4186,12 +4234,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Sebastian</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Medina</t>
+          <t>Diaby</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -4201,7 +4249,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>STU</t>
         </is>
       </c>
       <c r="E61" t="n">
@@ -4214,13 +4262,13 @@
         <v>0</v>
       </c>
       <c r="H61" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="I61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K61" t="n">
         <v>0</v>
@@ -4229,31 +4277,31 @@
         <v>0</v>
       </c>
       <c r="M61" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Sebastian</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Quansah</t>
+          <t>Neuer</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Leverkusen</t>
+          <t>Bayern</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E62" t="n">
@@ -4275,56 +4323,56 @@
         <v>0</v>
       </c>
       <c r="K62" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L62" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M62" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N62" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Sebastian</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Avdullahu</t>
+          <t>Urbig</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Hoffenheim</t>
+          <t>Bayern</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E63" t="n">
         <v>1</v>
       </c>
       <c r="F63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G63" t="n">
         <v>0</v>
       </c>
       <c r="H63" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K63" t="n">
         <v>0</v>
@@ -4333,7 +4381,7 @@
         <v>0</v>
       </c>
       <c r="M63" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N63" t="n">
         <v>0</v>
@@ -4347,21 +4395,21 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Führich</t>
+          <t>Anton</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Stuttgart</t>
+          <t>Dortmund</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F64" t="n">
         <v>0</v>
@@ -4370,7 +4418,7 @@
         <v>0</v>
       </c>
       <c r="H64" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -4379,13 +4427,13 @@
         <v>0</v>
       </c>
       <c r="K64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M64" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N64" t="n">
         <v>0</v>
@@ -4399,21 +4447,21 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Kai. Sano</t>
+          <t>Medina</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Mainz</t>
+          <t>Leverkusen</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F65" t="n">
         <v>0</v>
@@ -4422,13 +4470,13 @@
         <v>0</v>
       </c>
       <c r="H65" t="n">
-        <v>3.5</v>
+        <v>2.33</v>
       </c>
       <c r="I65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K65" t="n">
         <v>0</v>
@@ -4437,10 +4485,10 @@
         <v>0</v>
       </c>
       <c r="M65" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66">
@@ -4451,21 +4499,21 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Khedira</t>
+          <t>Quansah</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Union</t>
+          <t>Leverkusen</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E66" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F66" t="n">
         <v>0</v>
@@ -4474,7 +4522,7 @@
         <v>0</v>
       </c>
       <c r="H66" t="n">
-        <v>4.5</v>
+        <v>2.67</v>
       </c>
       <c r="I66" t="n">
         <v>0</v>
@@ -4483,16 +4531,16 @@
         <v>0</v>
       </c>
       <c r="K66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M66" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67">
@@ -4503,21 +4551,21 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>M. Eggestein</t>
+          <t>R. Koch</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Freiburg</t>
+          <t>Frankfurt</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E67" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F67" t="n">
         <v>0</v>
@@ -4526,22 +4574,22 @@
         <v>0</v>
       </c>
       <c r="H67" t="n">
-        <v>2.5</v>
+        <v>4.5</v>
       </c>
       <c r="I67" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J67" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M67" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N67" t="n">
         <v>0</v>
@@ -4555,12 +4603,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Musiala</t>
+          <t>Avdullahu</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Hoffenheim</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -4578,13 +4626,13 @@
         <v>0</v>
       </c>
       <c r="H68" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K68" t="n">
         <v>0</v>
@@ -4607,12 +4655,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Petkov</t>
+          <t>Führich</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Elversberg</t>
+          <t>Stuttgart</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -4621,7 +4669,7 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F69" t="n">
         <v>0</v>
@@ -4630,7 +4678,7 @@
         <v>0</v>
       </c>
       <c r="H69" t="n">
-        <v>2.5</v>
+        <v>3.75</v>
       </c>
       <c r="I69" t="n">
         <v>0</v>
@@ -4639,10 +4687,10 @@
         <v>0</v>
       </c>
       <c r="K69" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L69" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M69" t="n">
         <v>0</v>
@@ -4659,12 +4707,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Prömel</t>
+          <t>Kai. Sano</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Stuttgart</t>
+          <t>Mainz</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -4673,7 +4721,7 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F70" t="n">
         <v>0</v>
@@ -4682,13 +4730,13 @@
         <v>0</v>
       </c>
       <c r="H70" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="I70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K70" t="n">
         <v>0</v>
@@ -4711,17 +4759,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Ebnoutalib</t>
+          <t>Khedira</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Frankfurt</t>
+          <t>Union</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>STU</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E71" t="n">
@@ -4743,10 +4791,10 @@
         <v>0</v>
       </c>
       <c r="K71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M71" t="n">
         <v>0</v>
@@ -4763,21 +4811,21 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Schick</t>
+          <t>M. Eggestein</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Leverkusen</t>
+          <t>Freiburg</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>STU</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E72" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F72" t="n">
         <v>0</v>
@@ -4786,19 +4834,19 @@
         <v>0</v>
       </c>
       <c r="H72" t="n">
-        <v>1.75</v>
+        <v>2.83</v>
       </c>
       <c r="I72" t="n">
         <v>2</v>
       </c>
       <c r="J72" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K72" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L72" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M72" t="n">
         <v>0</v>
@@ -4815,17 +4863,17 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Undav</t>
+          <t>Moore</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Stuttgart</t>
+          <t>Köln</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>STU</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E73" t="n">
@@ -4838,7 +4886,7 @@
         <v>0</v>
       </c>
       <c r="H73" t="n">
-        <v>5</v>
+        <v>3.5</v>
       </c>
       <c r="I73" t="n">
         <v>0</v>
@@ -4867,17 +4915,17 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Atubolu</t>
+          <t>Musiala</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Frankfurt</t>
+          <t>Bayern</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E74" t="n">
@@ -4890,22 +4938,22 @@
         <v>0</v>
       </c>
       <c r="H74" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="I74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L74" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M74" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="N74" t="n">
         <v>0</v>
@@ -4914,50 +4962,50 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Wolfgang</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Baku</t>
+          <t>Petkov</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Leipzig</t>
+          <t>Elversberg</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E75" t="n">
         <v>2</v>
       </c>
       <c r="F75" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G75" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H75" t="n">
-        <v>4.5</v>
+        <v>3.25</v>
       </c>
       <c r="I75" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J75" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L75" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M75" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="N75" t="n">
         <v>0</v>
@@ -4966,26 +5014,26 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Wolfgang</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Brown</t>
+          <t>Prömel</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Stuttgart</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F76" t="n">
         <v>0</v>
@@ -4994,13 +5042,13 @@
         <v>0</v>
       </c>
       <c r="H76" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="I76" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J76" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K76" t="n">
         <v>0</v>
@@ -5018,22 +5066,22 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Wolfgang</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Schlotterbeck</t>
+          <t>Ebnoutalib</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Dortmund</t>
+          <t>Frankfurt</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>STU</t>
         </is>
       </c>
       <c r="E77" t="n">
@@ -5046,7 +5094,7 @@
         <v>0</v>
       </c>
       <c r="H77" t="n">
-        <v>2.5</v>
+        <v>4.5</v>
       </c>
       <c r="I77" t="n">
         <v>0</v>
@@ -5055,10 +5103,10 @@
         <v>0</v>
       </c>
       <c r="K77" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L77" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M77" t="n">
         <v>0</v>
@@ -5070,22 +5118,22 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Wolfgang</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Svensson</t>
+          <t>Hlozek</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Dortmund</t>
+          <t>Hoffenheim</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>STU</t>
         </is>
       </c>
       <c r="E78" t="n">
@@ -5098,7 +5146,7 @@
         <v>0</v>
       </c>
       <c r="H78" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="I78" t="n">
         <v>0</v>
@@ -5122,26 +5170,26 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Wolfgang</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Tah</t>
+          <t>Schick</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Leverkusen</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>ABW</t>
+          <t>STU</t>
         </is>
       </c>
       <c r="E79" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F79" t="n">
         <v>0</v>
@@ -5150,19 +5198,19 @@
         <v>0</v>
       </c>
       <c r="H79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I79" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J79" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="K79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M79" t="n">
         <v>0</v>
@@ -5174,22 +5222,22 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Wolfgang</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>El Aynaoui</t>
+          <t>Undav</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Leipzig</t>
+          <t>Stuttgart</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>STU</t>
         </is>
       </c>
       <c r="E80" t="n">
@@ -5202,7 +5250,7 @@
         <v>0</v>
       </c>
       <c r="H80" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I80" t="n">
         <v>0</v>
@@ -5226,26 +5274,26 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Wolfgang</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Fabio Vieira</t>
+          <t>Atubolu</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>HSV</t>
+          <t>Frankfurt</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E81" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F81" t="n">
         <v>0</v>
@@ -5254,7 +5302,7 @@
         <v>0</v>
       </c>
       <c r="H81" t="n">
-        <v>5</v>
+        <v>3.5</v>
       </c>
       <c r="I81" t="n">
         <v>0</v>
@@ -5269,7 +5317,7 @@
         <v>0</v>
       </c>
       <c r="M81" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="N81" t="n">
         <v>0</v>
@@ -5283,45 +5331,45 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Honorat</t>
+          <t>Baku</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Gladbach</t>
+          <t>Leipzig</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E82" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F82" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G82" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H82" t="n">
-        <v>2.5</v>
+        <v>4.5</v>
       </c>
       <c r="I82" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J82" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K82" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L82" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M82" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N82" t="n">
         <v>0</v>
@@ -5335,21 +5383,21 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Lee</t>
+          <t>Brown</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Mainz</t>
+          <t>Bayern</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E83" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F83" t="n">
         <v>0</v>
@@ -5367,10 +5415,10 @@
         <v>0</v>
       </c>
       <c r="K83" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L83" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M83" t="n">
         <v>0</v>
@@ -5387,21 +5435,21 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Nwaneri</t>
+          <t>Kabak</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Dortmund</t>
+          <t>Hoffenheim</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E84" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F84" t="n">
         <v>0</v>
@@ -5410,7 +5458,7 @@
         <v>0</v>
       </c>
       <c r="H84" t="n">
-        <v>3.25</v>
+        <v>4.5</v>
       </c>
       <c r="I84" t="n">
         <v>0</v>
@@ -5419,13 +5467,13 @@
         <v>0</v>
       </c>
       <c r="K84" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L84" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M84" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N84" t="n">
         <v>0</v>
@@ -5439,17 +5487,17 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Suzuki</t>
+          <t>Schlotterbeck</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Freiburg</t>
+          <t>Dortmund</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E85" t="n">
@@ -5462,7 +5510,7 @@
         <v>0</v>
       </c>
       <c r="H85" t="n">
-        <v>3.75</v>
+        <v>2.5</v>
       </c>
       <c r="I85" t="n">
         <v>0</v>
@@ -5491,7 +5539,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Veerman</t>
+          <t>Svensson</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -5501,7 +5549,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E86" t="n">
@@ -5514,7 +5562,7 @@
         <v>0</v>
       </c>
       <c r="H86" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="I86" t="n">
         <v>0</v>
@@ -5543,21 +5591,21 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Füllkrug</t>
+          <t>Tah</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Bremen</t>
+          <t>Bayern</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>STU</t>
+          <t>ABW</t>
         </is>
       </c>
       <c r="E87" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F87" t="n">
         <v>0</v>
@@ -5566,13 +5614,13 @@
         <v>0</v>
       </c>
       <c r="H87" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="I87" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J87" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K87" t="n">
         <v>0</v>
@@ -5595,21 +5643,21 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Luis Diaz</t>
+          <t>El Aynaoui</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Leipzig</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>STU</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E88" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F88" t="n">
         <v>0</v>
@@ -5618,7 +5666,7 @@
         <v>0</v>
       </c>
       <c r="H88" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I88" t="n">
         <v>0</v>
@@ -5647,17 +5695,17 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Mokwa</t>
+          <t>Fabio Vieira</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Elversberg</t>
+          <t>HSV</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>STU</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E89" t="n">
@@ -5670,13 +5718,13 @@
         <v>0</v>
       </c>
       <c r="H89" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I89" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J89" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K89" t="n">
         <v>0</v>
@@ -5699,21 +5747,21 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Saibari</t>
+          <t>Honorat</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Gladbach</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>STU</t>
+          <t>MIT</t>
         </is>
       </c>
       <c r="E90" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F90" t="n">
         <v>0</v>
@@ -5731,10 +5779,10 @@
         <v>0</v>
       </c>
       <c r="K90" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L90" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M90" t="n">
         <v>0</v>
@@ -5751,52 +5799,468 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
+          <t>Lee</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Mainz</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>3</v>
+      </c>
+      <c r="F91" t="n">
+        <v>0</v>
+      </c>
+      <c r="G91" t="n">
+        <v>0</v>
+      </c>
+      <c r="H91" t="n">
+        <v>4</v>
+      </c>
+      <c r="I91" t="n">
+        <v>0</v>
+      </c>
+      <c r="J91" t="n">
+        <v>0</v>
+      </c>
+      <c r="K91" t="n">
+        <v>1</v>
+      </c>
+      <c r="L91" t="n">
+        <v>2</v>
+      </c>
+      <c r="M91" t="n">
+        <v>0</v>
+      </c>
+      <c r="N91" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Wolfgang</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Nwaneri</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>2</v>
+      </c>
+      <c r="F92" t="n">
+        <v>0</v>
+      </c>
+      <c r="G92" t="n">
+        <v>0</v>
+      </c>
+      <c r="H92" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="I92" t="n">
+        <v>0</v>
+      </c>
+      <c r="J92" t="n">
+        <v>0</v>
+      </c>
+      <c r="K92" t="n">
+        <v>1</v>
+      </c>
+      <c r="L92" t="n">
+        <v>2</v>
+      </c>
+      <c r="M92" t="n">
+        <v>0</v>
+      </c>
+      <c r="N92" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Wolfgang</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Suzuki</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Freiburg</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>3</v>
+      </c>
+      <c r="F93" t="n">
+        <v>0</v>
+      </c>
+      <c r="G93" t="n">
+        <v>0</v>
+      </c>
+      <c r="H93" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="I93" t="n">
+        <v>1</v>
+      </c>
+      <c r="J93" t="n">
+        <v>1</v>
+      </c>
+      <c r="K93" t="n">
+        <v>0</v>
+      </c>
+      <c r="L93" t="n">
+        <v>0</v>
+      </c>
+      <c r="M93" t="n">
+        <v>0</v>
+      </c>
+      <c r="N93" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Wolfgang</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Veerman</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>2</v>
+      </c>
+      <c r="F94" t="n">
+        <v>0</v>
+      </c>
+      <c r="G94" t="n">
+        <v>0</v>
+      </c>
+      <c r="H94" t="n">
+        <v>3</v>
+      </c>
+      <c r="I94" t="n">
+        <v>0</v>
+      </c>
+      <c r="J94" t="n">
+        <v>0</v>
+      </c>
+      <c r="K94" t="n">
+        <v>0</v>
+      </c>
+      <c r="L94" t="n">
+        <v>0</v>
+      </c>
+      <c r="M94" t="n">
+        <v>0</v>
+      </c>
+      <c r="N94" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Wolfgang</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Füllkrug</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Bremen</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>STU</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>2</v>
+      </c>
+      <c r="F95" t="n">
+        <v>0</v>
+      </c>
+      <c r="G95" t="n">
+        <v>0</v>
+      </c>
+      <c r="H95" t="n">
+        <v>2</v>
+      </c>
+      <c r="I95" t="n">
+        <v>2</v>
+      </c>
+      <c r="J95" t="n">
+        <v>4</v>
+      </c>
+      <c r="K95" t="n">
+        <v>0</v>
+      </c>
+      <c r="L95" t="n">
+        <v>0</v>
+      </c>
+      <c r="M95" t="n">
+        <v>0</v>
+      </c>
+      <c r="N95" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Wolfgang</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Luis Diaz</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Bayern</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>STU</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>2</v>
+      </c>
+      <c r="F96" t="n">
+        <v>0</v>
+      </c>
+      <c r="G96" t="n">
+        <v>0</v>
+      </c>
+      <c r="H96" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="I96" t="n">
+        <v>0</v>
+      </c>
+      <c r="J96" t="n">
+        <v>0</v>
+      </c>
+      <c r="K96" t="n">
+        <v>0</v>
+      </c>
+      <c r="L96" t="n">
+        <v>0</v>
+      </c>
+      <c r="M96" t="n">
+        <v>0</v>
+      </c>
+      <c r="N96" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Wolfgang</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Mokwa</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Elversberg</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>STU</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>1</v>
+      </c>
+      <c r="F97" t="n">
+        <v>0</v>
+      </c>
+      <c r="G97" t="n">
+        <v>0</v>
+      </c>
+      <c r="H97" t="n">
+        <v>2</v>
+      </c>
+      <c r="I97" t="n">
+        <v>1</v>
+      </c>
+      <c r="J97" t="n">
+        <v>2</v>
+      </c>
+      <c r="K97" t="n">
+        <v>0</v>
+      </c>
+      <c r="L97" t="n">
+        <v>0</v>
+      </c>
+      <c r="M97" t="n">
+        <v>0</v>
+      </c>
+      <c r="N97" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Wolfgang</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Saibari</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Bayern</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>STU</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>1</v>
+      </c>
+      <c r="F98" t="n">
+        <v>0</v>
+      </c>
+      <c r="G98" t="n">
+        <v>0</v>
+      </c>
+      <c r="H98" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I98" t="n">
+        <v>0</v>
+      </c>
+      <c r="J98" t="n">
+        <v>0</v>
+      </c>
+      <c r="K98" t="n">
+        <v>1</v>
+      </c>
+      <c r="L98" t="n">
+        <v>1</v>
+      </c>
+      <c r="M98" t="n">
+        <v>0</v>
+      </c>
+      <c r="N98" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Wolfgang</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
           <t>Vandevoordt</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr">
+      <c r="C99" t="inlineStr">
         <is>
           <t>Leipzig</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr">
+      <c r="D99" t="inlineStr">
         <is>
           <t>TOR</t>
         </is>
       </c>
-      <c r="E91" t="n">
-        <v>2</v>
-      </c>
-      <c r="F91" t="n">
-        <v>0</v>
-      </c>
-      <c r="G91" t="n">
-        <v>0</v>
-      </c>
-      <c r="H91" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="I91" t="n">
-        <v>0</v>
-      </c>
-      <c r="J91" t="n">
-        <v>0</v>
-      </c>
-      <c r="K91" t="n">
-        <v>0</v>
-      </c>
-      <c r="L91" t="n">
-        <v>0</v>
-      </c>
-      <c r="M91" t="n">
-        <v>6</v>
-      </c>
-      <c r="N91" t="n">
+      <c r="E99" t="n">
+        <v>3</v>
+      </c>
+      <c r="F99" t="n">
+        <v>0</v>
+      </c>
+      <c r="G99" t="n">
+        <v>0</v>
+      </c>
+      <c r="H99" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="I99" t="n">
+        <v>0</v>
+      </c>
+      <c r="J99" t="n">
+        <v>0</v>
+      </c>
+      <c r="K99" t="n">
+        <v>0</v>
+      </c>
+      <c r="L99" t="n">
+        <v>0</v>
+      </c>
+      <c r="M99" t="n">
+        <v>10</v>
+      </c>
+      <c r="N99" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N91"/>
+  <autoFilter ref="A1:N99"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>